<commit_message>
feat: Bổ sung module Native VBA và xử lý chuẩn lũy kế Quý 2 cho BCTC hợp nhất
</commit_message>
<xml_diff>
--- a/templates/Mau_BCTC_Hop_Nhat_TCTD.xlsx
+++ b/templates/Mau_BCTC_Hop_Nhat_TCTD.xlsx
@@ -6,27 +6,28 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4275" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="B02" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="B03" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="B04" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="B05" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Thue" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TSCD2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="so lieu" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="But toan can tru" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Sổ chi tiết TK LN" sheetId="9" state="hidden" r:id="rId9"/>
-    <sheet name="Thuế TNDN Q4" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="TRANG_CHU" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="B02" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="B03" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="B04" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="B05" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Thue" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TSCD2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="so lieu" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="But toan can tru" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Sổ chi tiết TK LN" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet name="Thuế TNDN Q4" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId11"/>
     <externalReference r:id="rId12"/>
     <externalReference r:id="rId13"/>
     <externalReference r:id="rId14"/>
     <externalReference r:id="rId15"/>
+    <externalReference r:id="rId16"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TSCD2025'!$A$3:$S$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'so lieu'!$K$1:$P$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'TSCD2025'!$A$3:$S$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'so lieu'!$K$1:$P$87</definedName>
   </definedNames>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
@@ -159,7 +160,7 @@
     <numFmt numFmtId="285" formatCode="_-&quot;F&quot;* #,##0_-;\-&quot;F&quot;* #,##0_-;_-&quot;F&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="286" formatCode="_-&quot;F&quot;* ###,0&quot;$&quot;00_-;\-&quot;F&quot;* ###,0&quot;$&quot;00_-;_-&quot;F&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="203">
+  <fonts count="214">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1354,8 +1355,71 @@
       <color rgb="FF808080"/>
       <sz val="5"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001B365D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00002060"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="41">
     <fill>
       <patternFill/>
     </fill>
@@ -1549,6 +1613,48 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF0F0F0"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B365D"/>
+        <bgColor rgb="001B365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5597"/>
+        <bgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+        <bgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00333f48"/>
+        <bgColor rgb="00333f48"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -3703,7 +3809,7 @@
     <xf numFmtId="0" fontId="195" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="698">
+  <cellXfs count="716">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -5418,6 +5524,46 @@
     <xf numFmtId="167" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="170" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="43" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="203" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="204" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="205" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="206" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="207" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="208" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="209" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="210" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="207" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="211" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="212" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="210" fillId="39" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="213" fillId="40" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="213" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="769">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9185,6 +9331,1152 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" style="373" min="1" max="1"/>
+    <col width="35" customWidth="1" style="373" min="2" max="2"/>
+    <col width="25" customWidth="1" style="373" min="3" max="3"/>
+    <col width="25" customWidth="1" style="373" min="4" max="4"/>
+    <col width="25" customWidth="1" style="373" min="5" max="5"/>
+    <col width="28" customWidth="1" style="373" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="698" t="inlineStr">
+        <is>
+          <t>BỘ CÔNG CỤ LẬP BÁO CÁO TÀI CHÍNH PHỤC VỤ HỢP NHẤT
+(CHUẨN KẾ TOÁN TỔ CHỨC TÍN DỤNG - TCTD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="5">
+      <c r="B5" s="700" t="inlineStr">
+        <is>
+          <t>📁 BƯỚC 1: CHỌN FILE BẢNG CÂN ĐỐI TÀI KHOẢN (TT200)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="701" t="inlineStr">
+        <is>
+          <t>1.1. Bấm nút macro:</t>
+        </is>
+      </c>
+      <c r="C6" s="702" t="inlineStr">
+        <is>
+          <t>👉 [ BẤM ĐỂ CHỌN FILE CĐTK ] (Macro: ChonFileBangCanDoi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="703" t="inlineStr">
+        <is>
+          <t>1.2. Đường dẫn file:</t>
+        </is>
+      </c>
+      <c r="C7" s="704" t="inlineStr">
+        <is>
+          <t>data/Bang_can_doi_tai_khoanQ22026.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="703" t="inlineStr">
+        <is>
+          <t>1.3. Kỳ kế toán nhận diện:</t>
+        </is>
+      </c>
+      <c r="C8" s="705" t="inlineStr">
+        <is>
+          <t>QUÝ 2 NĂM 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="700" t="inlineStr">
+        <is>
+          <t>⚙️ BƯỚC 2: CẤU HÌNH BÚT TOÁN CẤN TRỪ (Intercompany Elimination)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="706" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="C12" s="706" t="inlineStr">
+        <is>
+          <t>Tên bút toán cấn trừ / điều chỉnh</t>
+        </is>
+      </c>
+      <c r="D12" s="706" t="inlineStr">
+        <is>
+          <t>Tự động gợi ý (VND)</t>
+        </is>
+      </c>
+      <c r="E12" s="706" t="inlineStr">
+        <is>
+          <t>Sửa thủ công (nếu có)</t>
+        </is>
+      </c>
+      <c r="F12" s="706" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="707" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Cấn trừ trung gian ngoại tệ (TK 33886.02 / 13885.02)</t>
+        </is>
+      </c>
+      <c r="D13" s="708" t="n">
+        <v>10460694846</v>
+      </c>
+      <c r="E13" s="709" t="inlineStr"/>
+      <c r="F13" s="710" t="inlineStr">
+        <is>
+          <t>Tự lấy số dư CK TK 13885.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="707" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Chuyển phải thu NHCT về tiền gửi (TK 11211.01 / 13881)</t>
+        </is>
+      </c>
+      <c r="D14" s="708" t="n">
+        <v>18358019545</v>
+      </c>
+      <c r="E14" s="709" t="inlineStr"/>
+      <c r="F14" s="710" t="inlineStr">
+        <is>
+          <t>Tự lấy số dư CK TK 13881</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="707" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Cấn trừ đối tác Western Union (WU) (TK 33882.01 / 13882.02)</t>
+        </is>
+      </c>
+      <c r="D15" s="708" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="709" t="inlineStr"/>
+      <c r="F15" s="710" t="inlineStr">
+        <is>
+          <t>Mặc định 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="707" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Cấn trừ các tài khoản WASH (TK 33883.01 / 1121)</t>
+        </is>
+      </c>
+      <c r="D16" s="708" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="709" t="inlineStr"/>
+      <c r="F16" s="710" t="inlineStr">
+        <is>
+          <t>Mặc định 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="700" t="inlineStr">
+        <is>
+          <t>⚡ BƯỚC 3: CẬP NHẬT SỐ LIỆU &amp; LẬP BÁO CÁO HỢP NHẤT</t>
+        </is>
+      </c>
+      <c r="C18" s="711" t="inlineStr">
+        <is>
+          <t>👉 [ BẤM ĐỂ LẬP BÁO CÁO HỢP NHẤT ] (Macro: CapNhatVaLapBaoCaoHopNhat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="700" t="inlineStr">
+        <is>
+          <t>📊 KẾT QUẢ KIỂM TRA TÍNH CÂN ĐỐI (STATUS DASHBOARD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="712" t="inlineStr">
+        <is>
+          <t>Chỉ tiêu đối chiếu</t>
+        </is>
+      </c>
+      <c r="C21" s="712" t="inlineStr">
+        <is>
+          <t>Tổng Nợ (VNĐ)</t>
+        </is>
+      </c>
+      <c r="D21" s="712" t="inlineStr">
+        <is>
+          <t>Tổng Có (VNĐ)</t>
+        </is>
+      </c>
+      <c r="E21" s="712" t="inlineStr">
+        <is>
+          <t>Trạng thái cân đối</t>
+        </is>
+      </c>
+      <c r="F21" s="712" t="inlineStr">
+        <is>
+          <t>Đánh giá</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="703" t="inlineStr">
+        <is>
+          <t>1. Số dư Đầu kỳ (Sheet so lieu)</t>
+        </is>
+      </c>
+      <c r="C22" s="713" t="n">
+        <v>231464686791</v>
+      </c>
+      <c r="D22" s="713" t="n">
+        <v>231464686791</v>
+      </c>
+      <c r="E22" s="714" t="inlineStr">
+        <is>
+          <t>CÂN ĐỐI (0 đ)</t>
+        </is>
+      </c>
+      <c r="F22" s="715" t="inlineStr">
+        <is>
+          <t>✅ Hoàn hảo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="703" t="inlineStr">
+        <is>
+          <t>2. Phát sinh trong kỳ (Sheet so lieu)</t>
+        </is>
+      </c>
+      <c r="C23" s="713" t="n">
+        <v>52142209214992</v>
+      </c>
+      <c r="D23" s="713" t="n">
+        <v>52142209214992</v>
+      </c>
+      <c r="E23" s="714" t="inlineStr">
+        <is>
+          <t>CÂN ĐỐI (0 đ)</t>
+        </is>
+      </c>
+      <c r="F23" s="715" t="inlineStr">
+        <is>
+          <t>✅ Hoàn hảo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="703" t="inlineStr">
+        <is>
+          <t>3. Số dư Cuối kỳ (Sheet so lieu)</t>
+        </is>
+      </c>
+      <c r="C24" s="713" t="n">
+        <v>315725226474</v>
+      </c>
+      <c r="D24" s="713" t="n">
+        <v>315725226474</v>
+      </c>
+      <c r="E24" s="714" t="inlineStr">
+        <is>
+          <t>CÂN ĐỐI (0 đ)</t>
+        </is>
+      </c>
+      <c r="F24" s="715" t="inlineStr">
+        <is>
+          <t>✅ Hoàn hảo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="B2:F3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Sheet10">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="292" min="1" max="2"/>
+    <col width="10" customWidth="1" style="373" min="3" max="3"/>
+    <col width="29.28515625" bestFit="1" customWidth="1" style="373" min="4" max="4"/>
+    <col width="9.140625" customWidth="1" style="373" min="5" max="6"/>
+    <col width="14" bestFit="1" customWidth="1" style="315" min="7" max="7"/>
+    <col width="11.42578125" bestFit="1" customWidth="1" style="294" min="8" max="8"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" style="315" min="9" max="9"/>
+    <col width="11.42578125" bestFit="1" customWidth="1" style="294" min="10" max="10"/>
+    <col width="5.42578125" bestFit="1" customWidth="1" style="315" min="11" max="11"/>
+    <col width="5.5703125" bestFit="1" customWidth="1" style="294" min="12" max="12"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" style="315" min="13" max="13"/>
+    <col width="11.42578125" bestFit="1" customWidth="1" style="294" min="14" max="14"/>
+    <col width="13.5703125" customWidth="1" style="373" min="15" max="15"/>
+    <col width="18.140625" customWidth="1" style="373" min="16" max="16"/>
+    <col width="8.7109375" customWidth="1" style="373" min="17" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18.75" customHeight="1" s="373">
+      <c r="A1" s="516" t="inlineStr">
+        <is>
+          <t>SỔ CHI TIẾT CÁC TÀI KHOẢN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="517" t="inlineStr">
+        <is>
+          <t>Loại tiền: Tổng hợp; Tài khoản: 421; Quý 1 năm 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="373">
+      <c r="A3" s="522" t="inlineStr">
+        <is>
+          <t>Ngày hạch toán</t>
+        </is>
+      </c>
+      <c r="B3" s="522" t="inlineStr">
+        <is>
+          <t>Ngày chứng từ</t>
+        </is>
+      </c>
+      <c r="C3" s="518" t="inlineStr">
+        <is>
+          <t>Số chứng từ</t>
+        </is>
+      </c>
+      <c r="D3" s="518" t="inlineStr">
+        <is>
+          <t>Diễn giải</t>
+        </is>
+      </c>
+      <c r="E3" s="518" t="inlineStr">
+        <is>
+          <t>Tài khoản</t>
+        </is>
+      </c>
+      <c r="F3" s="518" t="inlineStr">
+        <is>
+          <t>TK đối ứng</t>
+        </is>
+      </c>
+      <c r="G3" s="683" t="inlineStr">
+        <is>
+          <t>Phát sinh Nợ</t>
+        </is>
+      </c>
+      <c r="H3" s="684" t="n"/>
+      <c r="I3" s="683" t="inlineStr">
+        <is>
+          <t>Phát sinh Có</t>
+        </is>
+      </c>
+      <c r="J3" s="684" t="n"/>
+      <c r="K3" s="683" t="inlineStr">
+        <is>
+          <t>Dư Nợ</t>
+        </is>
+      </c>
+      <c r="L3" s="684" t="n"/>
+      <c r="M3" s="683" t="inlineStr">
+        <is>
+          <t>Dư Có</t>
+        </is>
+      </c>
+      <c r="N3" s="684" t="n"/>
+      <c r="O3" s="518" t="inlineStr">
+        <is>
+          <t>Mã mục thu/chi</t>
+        </is>
+      </c>
+      <c r="P3" s="518" t="inlineStr">
+        <is>
+          <t>Tên mục thu/chi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="373">
+      <c r="A4" s="685" t="n"/>
+      <c r="B4" s="685" t="n"/>
+      <c r="C4" s="685" t="n"/>
+      <c r="D4" s="685" t="n"/>
+      <c r="E4" s="685" t="n"/>
+      <c r="F4" s="685" t="n"/>
+      <c r="G4" s="376" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="H4" s="377" t="inlineStr">
+        <is>
+          <t>Quy đổi</t>
+        </is>
+      </c>
+      <c r="I4" s="376" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="J4" s="377" t="inlineStr">
+        <is>
+          <t>Quy đổi</t>
+        </is>
+      </c>
+      <c r="K4" s="376" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="L4" s="377" t="inlineStr">
+        <is>
+          <t>Quy đổi</t>
+        </is>
+      </c>
+      <c r="M4" s="376" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="N4" s="377" t="inlineStr">
+        <is>
+          <t>Quy đổi</t>
+        </is>
+      </c>
+      <c r="O4" s="685" t="n"/>
+      <c r="P4" s="685" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="378" t="n"/>
+      <c r="B5" s="378" t="n"/>
+      <c r="C5" s="379" t="inlineStr"/>
+      <c r="D5" s="379" t="inlineStr">
+        <is>
+          <t>Số dư đầu kỳ</t>
+        </is>
+      </c>
+      <c r="E5" s="379" t="inlineStr">
+        <is>
+          <t>421</t>
+        </is>
+      </c>
+      <c r="F5" s="379" t="n"/>
+      <c r="G5" s="380" t="n"/>
+      <c r="H5" s="381" t="n"/>
+      <c r="I5" s="380" t="n"/>
+      <c r="J5" s="381" t="n"/>
+      <c r="K5" s="380" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="381" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="380" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="N5" s="381" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="O5" s="379" t="n"/>
+      <c r="P5" s="379" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="378" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B6" s="378" t="n">
+        <v>46027</v>
+      </c>
+      <c r="C6" s="379" t="inlineStr">
+        <is>
+          <t>ZKC01</t>
+        </is>
+      </c>
+      <c r="D6" s="379" t="inlineStr">
+        <is>
+          <t>Kết chuyển lợi nhuận sau thuế năm 2025</t>
+        </is>
+      </c>
+      <c r="E6" s="379" t="inlineStr">
+        <is>
+          <t>421</t>
+        </is>
+      </c>
+      <c r="F6" s="379" t="inlineStr">
+        <is>
+          <t>42121.01</t>
+        </is>
+      </c>
+      <c r="G6" s="380" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="381" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="380" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="J6" s="381" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="K6" s="380" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="381" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="380" t="n">
+        <v>35934868090</v>
+      </c>
+      <c r="N6" s="381" t="n">
+        <v>35934868090</v>
+      </c>
+      <c r="O6" s="379" t="n"/>
+      <c r="P6" s="379" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="378" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B7" s="378" t="n">
+        <v>46027</v>
+      </c>
+      <c r="C7" s="379" t="inlineStr">
+        <is>
+          <t>ZKC01</t>
+        </is>
+      </c>
+      <c r="D7" s="379" t="inlineStr">
+        <is>
+          <t>Kết chuyển lợi nhuận sau thuế năm 2025</t>
+        </is>
+      </c>
+      <c r="E7" s="379" t="inlineStr">
+        <is>
+          <t>421</t>
+        </is>
+      </c>
+      <c r="F7" s="379" t="inlineStr">
+        <is>
+          <t>42111.01</t>
+        </is>
+      </c>
+      <c r="G7" s="380" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="H7" s="381" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="I7" s="380" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="381" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="380" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="381" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="380" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="N7" s="381" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="O7" s="379" t="n"/>
+      <c r="P7" s="379" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="378" t="n"/>
+      <c r="B8" s="378" t="n"/>
+      <c r="C8" s="379" t="inlineStr"/>
+      <c r="D8" s="379" t="inlineStr">
+        <is>
+          <t>Cộng</t>
+        </is>
+      </c>
+      <c r="E8" s="379" t="inlineStr">
+        <is>
+          <t>421</t>
+        </is>
+      </c>
+      <c r="F8" s="379" t="n"/>
+      <c r="G8" s="380" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="H8" s="381" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="I8" s="380" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="J8" s="381" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="K8" s="380" t="n"/>
+      <c r="L8" s="381" t="n"/>
+      <c r="M8" s="380" t="n"/>
+      <c r="N8" s="381" t="n"/>
+      <c r="O8" s="379" t="n"/>
+      <c r="P8" s="379" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="378" t="n"/>
+      <c r="B9" s="378" t="n"/>
+      <c r="C9" s="379" t="inlineStr"/>
+      <c r="D9" s="379" t="inlineStr">
+        <is>
+          <t>Số dư cuối kỳ</t>
+        </is>
+      </c>
+      <c r="E9" s="379" t="inlineStr">
+        <is>
+          <t>421</t>
+        </is>
+      </c>
+      <c r="F9" s="379" t="n"/>
+      <c r="G9" s="380" t="n"/>
+      <c r="H9" s="381" t="n"/>
+      <c r="I9" s="380" t="n"/>
+      <c r="J9" s="381" t="n"/>
+      <c r="K9" s="380" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="381" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="380" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="N9" s="381" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="O9" s="379" t="n"/>
+      <c r="P9" s="379" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="382" t="inlineStr">
+        <is>
+          <t>Số dòng = 5</t>
+        </is>
+      </c>
+      <c r="G10" s="383" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="H10" s="384" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="I10" s="383" t="n">
+        <v>17967434045</v>
+      </c>
+      <c r="J10" s="384" t="n">
+        <v>17967434045</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="O3:O4"/>
+    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="I3:J3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <cols>
+    <col width="1.85546875" customWidth="1" style="352" min="1" max="1"/>
+    <col width="5.5703125" customWidth="1" style="352" min="2" max="2"/>
+    <col width="56.42578125" bestFit="1" customWidth="1" style="352" min="3" max="3"/>
+    <col width="23" customWidth="1" style="686" min="4" max="4"/>
+    <col width="34" customWidth="1" style="352" min="5" max="5"/>
+    <col width="20.42578125" bestFit="1" customWidth="1" style="352" min="6" max="6"/>
+    <col width="14.85546875" bestFit="1" customWidth="1" style="352" min="7" max="7"/>
+    <col width="34" customWidth="1" style="352" min="8" max="10"/>
+    <col width="9.140625" customWidth="1" style="352" min="11" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.75" customFormat="1" customHeight="1" s="338">
+      <c r="A1" s="336" t="inlineStr">
+        <is>
+          <t>Ten cong ty</t>
+        </is>
+      </c>
+      <c r="B1" s="336" t="n"/>
+      <c r="C1" s="687" t="n"/>
+      <c r="D1" s="336" t="n"/>
+      <c r="E1" s="336" t="n"/>
+    </row>
+    <row r="2" ht="15.75" customFormat="1" customHeight="1" s="338">
+      <c r="A2" s="336" t="inlineStr">
+        <is>
+          <t>PHÒNG TÀI CHÍNH KẾ TOÁN</t>
+        </is>
+      </c>
+      <c r="B2" s="336" t="n"/>
+      <c r="C2" s="687" t="n"/>
+      <c r="D2" s="336" t="n"/>
+      <c r="E2" s="336" t="n"/>
+    </row>
+    <row r="3" ht="15.75" customFormat="1" customHeight="1" s="338">
+      <c r="A3" s="336" t="n"/>
+      <c r="B3" s="336" t="n"/>
+      <c r="C3" s="687" t="n"/>
+      <c r="D3" s="336" t="n"/>
+      <c r="E3" s="336" t="n"/>
+    </row>
+    <row r="4" ht="32.25" customFormat="1" customHeight="1" s="338">
+      <c r="A4" s="524" t="inlineStr">
+        <is>
+          <t>BẢNG TÍNH THUẾ THU NHẬP DOANH NGHIỆP TẠM TÍNH Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="336" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" s="340" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="C6" s="340" t="inlineStr">
+        <is>
+          <t>Nội Dung</t>
+        </is>
+      </c>
+      <c r="D6" s="688" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Số tiền </t>
+        </is>
+      </c>
+      <c r="G6" s="689" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="340" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="340" t="inlineStr">
+        <is>
+          <t>Doanh thu Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D7" s="688">
+        <f>SUM(D8:D10)</f>
+        <v/>
+      </c>
+      <c r="G7" s="689" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="340" t="n"/>
+      <c r="C8" s="340" t="inlineStr">
+        <is>
+          <t>Doanh thu phí Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D8" s="688">
+        <f>[5]Sheet24!R31</f>
+        <v/>
+      </c>
+      <c r="G8" s="689" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="340" t="n"/>
+      <c r="C9" s="340" t="inlineStr">
+        <is>
+          <t>Doanh thu tài chính Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D9" s="688">
+        <f>[5]Sheet24!R32</f>
+        <v/>
+      </c>
+      <c r="F9" s="690" t="n"/>
+      <c r="G9" s="689" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="340" t="n"/>
+      <c r="C10" s="340" t="inlineStr">
+        <is>
+          <t>Thu nhập khác Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D10" s="688" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="340" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="340" t="inlineStr">
+        <is>
+          <t>Chi phí Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D11" s="688">
+        <f>SUM(D12:D16)</f>
+        <v/>
+      </c>
+      <c r="E11" s="691" t="inlineStr">
+        <is>
+          <t>Lợi nhuận trước thuế</t>
+        </is>
+      </c>
+      <c r="F11" s="692">
+        <f>D7-D11</f>
+        <v/>
+      </c>
+      <c r="G11" s="689" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="340" t="n"/>
+      <c r="C12" s="340" t="inlineStr">
+        <is>
+          <t>Giá vốn hàng bán Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D12" s="688">
+        <f>[5]Sheet24!P33</f>
+        <v/>
+      </c>
+      <c r="F12" s="690" t="n"/>
+      <c r="G12" s="689" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="340" t="n"/>
+      <c r="C13" s="340" t="inlineStr">
+        <is>
+          <t>Chi phí bán hàng Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D13" s="688" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="689" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="340" t="n"/>
+      <c r="C14" s="340" t="inlineStr">
+        <is>
+          <t>Chi phí tài chính Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D14" s="688">
+        <f>[5]Sheet24!J41</f>
+        <v/>
+      </c>
+      <c r="F14" s="693" t="n"/>
+      <c r="G14" s="689" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="340" t="n"/>
+      <c r="C15" s="340" t="inlineStr">
+        <is>
+          <t>Chi phí quản lý doanh nghiệp Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D15" s="694">
+        <f>[5]Sheet24!P42</f>
+        <v/>
+      </c>
+      <c r="G15" s="689" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="373">
+      <c r="B16" s="340" t="n"/>
+      <c r="C16" s="340" t="inlineStr">
+        <is>
+          <t>Chi phí khác</t>
+        </is>
+      </c>
+      <c r="D16" s="688">
+        <f>[5]Sheet24!M48</f>
+        <v/>
+      </c>
+      <c r="G16" s="689" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="340" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="340" t="inlineStr">
+        <is>
+          <t>Chi phí không được khấu trừ thuế TNDN Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D17" s="688">
+        <f>SUM(D18:D20)</f>
+        <v/>
+      </c>
+      <c r="G17" s="689" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="340" t="n"/>
+      <c r="C18" s="340" t="inlineStr">
+        <is>
+          <t>Chi thù lao chủ tịch + kiểm soát viên</t>
+        </is>
+      </c>
+      <c r="D18" s="688">
+        <f>15000000</f>
+        <v/>
+      </c>
+      <c r="G18" s="689" t="n"/>
+    </row>
+    <row r="19" hidden="1" s="373">
+      <c r="B19" s="340" t="n"/>
+      <c r="C19" s="340" t="inlineStr">
+        <is>
+          <t>Chi phí marketing khuyến mại giữ lại cho chi nhánh</t>
+        </is>
+      </c>
+      <c r="D19" s="688" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="373">
+      <c r="B20" s="340" t="n"/>
+      <c r="C20" s="340" t="inlineStr">
+        <is>
+          <t>Chi phí khác</t>
+        </is>
+      </c>
+      <c r="D20" s="688">
+        <f>[5]Sheet24!F48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="340" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="340" t="inlineStr">
+        <is>
+          <t>Chi phí tính thuế TNDN Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D21" s="688">
+        <f>D11-D17</f>
+        <v/>
+      </c>
+      <c r="E21" s="690" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="340" t="n">
+        <v>5</v>
+      </c>
+      <c r="C22" s="340" t="inlineStr">
+        <is>
+          <t>Thu nhập tính thuế thuế Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D22" s="688">
+        <f>D7-D21</f>
+        <v/>
+      </c>
+      <c r="E22" s="690" t="n"/>
+      <c r="F22" s="690" t="n"/>
+      <c r="G22" s="690" t="n"/>
+      <c r="H22" s="686" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="340" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" s="340" t="inlineStr">
+        <is>
+          <t>Thuế TNDN Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D23" s="688">
+        <f>ROUND(D22*0.2,0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="686" t="n"/>
+      <c r="G23" s="690" t="n"/>
+      <c r="H23" s="690" t="n"/>
+    </row>
+    <row r="24" hidden="1" s="373">
+      <c r="B24" s="340" t="n">
+        <v>7</v>
+      </c>
+      <c r="C24" s="340" t="inlineStr">
+        <is>
+          <t>Thuế TNDN quý 1.2024</t>
+        </is>
+      </c>
+      <c r="D24" s="688" t="n"/>
+      <c r="H24" s="695" t="n"/>
+    </row>
+    <row r="25" hidden="1" s="373">
+      <c r="B25" s="340" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" s="340" t="inlineStr">
+        <is>
+          <t>Thuế TNDN Quý 2.2024</t>
+        </is>
+      </c>
+      <c r="D25" s="688" t="n"/>
+      <c r="E25" s="693" t="n"/>
+      <c r="F25" s="693" t="n"/>
+    </row>
+    <row r="26" hidden="1" s="373">
+      <c r="B26" s="340" t="n">
+        <v>9</v>
+      </c>
+      <c r="C26" s="340" t="inlineStr">
+        <is>
+          <t>Thuế TNDN quý 3.2024</t>
+        </is>
+      </c>
+      <c r="D26" s="688" t="n"/>
+      <c r="E26" s="693" t="n"/>
+      <c r="F26" s="693" t="n"/>
+    </row>
+    <row r="27" hidden="1" s="373">
+      <c r="B27" s="340" t="n">
+        <v>10</v>
+      </c>
+      <c r="C27" s="340" t="inlineStr">
+        <is>
+          <t>Thuế TNDN quý 4.2024</t>
+        </is>
+      </c>
+      <c r="D27" s="696">
+        <f>D23-D24-D25-D26</f>
+        <v/>
+      </c>
+      <c r="E27" s="693" t="n"/>
+      <c r="F27" s="693" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="340" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" s="340" t="inlineStr">
+        <is>
+          <t>Lợi nhuận trước thuế</t>
+        </is>
+      </c>
+      <c r="D28" s="688">
+        <f>D7-D11</f>
+        <v/>
+      </c>
+      <c r="E28" s="693" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="340" t="n">
+        <v>8</v>
+      </c>
+      <c r="C29" s="340" t="inlineStr">
+        <is>
+          <t>Lợi nhuận sau thuế Quý 1 năm 2026</t>
+        </is>
+      </c>
+      <c r="D29" s="688">
+        <f>D28-D23</f>
+        <v/>
+      </c>
+      <c r="E29" s="693" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="352" t="n"/>
+      <c r="C30" s="352" t="n"/>
+      <c r="D30" s="686" t="n"/>
+      <c r="E30" s="693" t="n"/>
+      <c r="F30" s="693" t="n"/>
+      <c r="G30" s="697" t="n"/>
+      <c r="H30" s="697" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="525" t="inlineStr">
+        <is>
+          <t>Lập bảng                                         Kiểm soát                                              Tổng giám đốc</t>
+        </is>
+      </c>
+      <c r="H31" s="697" t="n"/>
+    </row>
+    <row r="32">
+      <c r="F32" s="690" t="n"/>
+    </row>
+    <row r="33">
+      <c r="F33" s="697" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="A4:D4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -11310,7 +12602,7 @@
       </c>
       <c r="C89" s="418" t="n"/>
       <c r="D89" s="540">
-        <f>'so lieu'!E41</f>
+        <f>'so lieu'!G41</f>
         <v/>
       </c>
       <c r="E89" s="540" t="n">
@@ -11849,443 +13141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H33"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
-  <cols>
-    <col width="1.85546875" customWidth="1" style="352" min="1" max="1"/>
-    <col width="5.5703125" customWidth="1" style="352" min="2" max="2"/>
-    <col width="56.42578125" bestFit="1" customWidth="1" style="352" min="3" max="3"/>
-    <col width="23" customWidth="1" style="686" min="4" max="4"/>
-    <col width="34" customWidth="1" style="352" min="5" max="5"/>
-    <col width="20.42578125" bestFit="1" customWidth="1" style="352" min="6" max="6"/>
-    <col width="14.85546875" bestFit="1" customWidth="1" style="352" min="7" max="7"/>
-    <col width="34" customWidth="1" style="352" min="8" max="10"/>
-    <col width="9.140625" customWidth="1" style="352" min="11" max="16384"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="15.75" customFormat="1" customHeight="1" s="338">
-      <c r="A1" s="336" t="inlineStr">
-        <is>
-          <t>Ten cong ty</t>
-        </is>
-      </c>
-      <c r="B1" s="336" t="n"/>
-      <c r="C1" s="687" t="n"/>
-      <c r="D1" s="336" t="n"/>
-      <c r="E1" s="336" t="n"/>
-    </row>
-    <row r="2" ht="15.75" customFormat="1" customHeight="1" s="338">
-      <c r="A2" s="336" t="inlineStr">
-        <is>
-          <t>PHÒNG TÀI CHÍNH KẾ TOÁN</t>
-        </is>
-      </c>
-      <c r="B2" s="336" t="n"/>
-      <c r="C2" s="687" t="n"/>
-      <c r="D2" s="336" t="n"/>
-      <c r="E2" s="336" t="n"/>
-    </row>
-    <row r="3" ht="15.75" customFormat="1" customHeight="1" s="338">
-      <c r="A3" s="336" t="n"/>
-      <c r="B3" s="336" t="n"/>
-      <c r="C3" s="687" t="n"/>
-      <c r="D3" s="336" t="n"/>
-      <c r="E3" s="336" t="n"/>
-    </row>
-    <row r="4" ht="32.25" customFormat="1" customHeight="1" s="338">
-      <c r="A4" s="524" t="inlineStr">
-        <is>
-          <t>BẢNG TÍNH THUẾ THU NHẬP DOANH NGHIỆP TẠM TÍNH Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="E4" s="336" t="n"/>
-    </row>
-    <row r="6">
-      <c r="B6" s="340" t="inlineStr">
-        <is>
-          <t>STT</t>
-        </is>
-      </c>
-      <c r="C6" s="340" t="inlineStr">
-        <is>
-          <t>Nội Dung</t>
-        </is>
-      </c>
-      <c r="D6" s="688" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Số tiền </t>
-        </is>
-      </c>
-      <c r="G6" s="689" t="n"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="340" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="340" t="inlineStr">
-        <is>
-          <t>Doanh thu Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D7" s="688">
-        <f>SUM(D8:D10)</f>
-        <v/>
-      </c>
-      <c r="G7" s="689" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="340" t="n"/>
-      <c r="C8" s="340" t="inlineStr">
-        <is>
-          <t>Doanh thu phí Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D8" s="688">
-        <f>[5]Sheet24!R31</f>
-        <v/>
-      </c>
-      <c r="G8" s="689" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="340" t="n"/>
-      <c r="C9" s="340" t="inlineStr">
-        <is>
-          <t>Doanh thu tài chính Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D9" s="688">
-        <f>[5]Sheet24!R32</f>
-        <v/>
-      </c>
-      <c r="F9" s="690" t="n"/>
-      <c r="G9" s="689" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="340" t="n"/>
-      <c r="C10" s="340" t="inlineStr">
-        <is>
-          <t>Thu nhập khác Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D10" s="688" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="340" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="340" t="inlineStr">
-        <is>
-          <t>Chi phí Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D11" s="688">
-        <f>SUM(D12:D16)</f>
-        <v/>
-      </c>
-      <c r="E11" s="691" t="inlineStr">
-        <is>
-          <t>Lợi nhuận trước thuế</t>
-        </is>
-      </c>
-      <c r="F11" s="692">
-        <f>D7-D11</f>
-        <v/>
-      </c>
-      <c r="G11" s="689" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="340" t="n"/>
-      <c r="C12" s="340" t="inlineStr">
-        <is>
-          <t>Giá vốn hàng bán Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D12" s="688">
-        <f>[5]Sheet24!P33</f>
-        <v/>
-      </c>
-      <c r="F12" s="690" t="n"/>
-      <c r="G12" s="689" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="340" t="n"/>
-      <c r="C13" s="340" t="inlineStr">
-        <is>
-          <t>Chi phí bán hàng Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D13" s="688" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="689" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="340" t="n"/>
-      <c r="C14" s="340" t="inlineStr">
-        <is>
-          <t>Chi phí tài chính Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D14" s="688">
-        <f>[5]Sheet24!J41</f>
-        <v/>
-      </c>
-      <c r="F14" s="693" t="n"/>
-      <c r="G14" s="689" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="340" t="n"/>
-      <c r="C15" s="340" t="inlineStr">
-        <is>
-          <t>Chi phí quản lý doanh nghiệp Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D15" s="694">
-        <f>[5]Sheet24!P42</f>
-        <v/>
-      </c>
-      <c r="G15" s="689" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="373">
-      <c r="B16" s="340" t="n"/>
-      <c r="C16" s="340" t="inlineStr">
-        <is>
-          <t>Chi phí khác</t>
-        </is>
-      </c>
-      <c r="D16" s="688">
-        <f>[5]Sheet24!M48</f>
-        <v/>
-      </c>
-      <c r="G16" s="689" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="340" t="n">
-        <v>3</v>
-      </c>
-      <c r="C17" s="340" t="inlineStr">
-        <is>
-          <t>Chi phí không được khấu trừ thuế TNDN Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D17" s="688">
-        <f>SUM(D18:D20)</f>
-        <v/>
-      </c>
-      <c r="G17" s="689" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="340" t="n"/>
-      <c r="C18" s="340" t="inlineStr">
-        <is>
-          <t>Chi thù lao chủ tịch + kiểm soát viên</t>
-        </is>
-      </c>
-      <c r="D18" s="688">
-        <f>15000000</f>
-        <v/>
-      </c>
-      <c r="G18" s="689" t="n"/>
-    </row>
-    <row r="19" hidden="1" s="373">
-      <c r="B19" s="340" t="n"/>
-      <c r="C19" s="340" t="inlineStr">
-        <is>
-          <t>Chi phí marketing khuyến mại giữ lại cho chi nhánh</t>
-        </is>
-      </c>
-      <c r="D19" s="688" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="373">
-      <c r="B20" s="340" t="n"/>
-      <c r="C20" s="340" t="inlineStr">
-        <is>
-          <t>Chi phí khác</t>
-        </is>
-      </c>
-      <c r="D20" s="688">
-        <f>[5]Sheet24!F48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="340" t="n">
-        <v>4</v>
-      </c>
-      <c r="C21" s="340" t="inlineStr">
-        <is>
-          <t>Chi phí tính thuế TNDN Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D21" s="688">
-        <f>D11-D17</f>
-        <v/>
-      </c>
-      <c r="E21" s="690" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="340" t="n">
-        <v>5</v>
-      </c>
-      <c r="C22" s="340" t="inlineStr">
-        <is>
-          <t>Thu nhập tính thuế thuế Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D22" s="688">
-        <f>D7-D21</f>
-        <v/>
-      </c>
-      <c r="E22" s="690" t="n"/>
-      <c r="F22" s="690" t="n"/>
-      <c r="G22" s="690" t="n"/>
-      <c r="H22" s="686" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="340" t="n">
-        <v>6</v>
-      </c>
-      <c r="C23" s="340" t="inlineStr">
-        <is>
-          <t>Thuế TNDN Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D23" s="688">
-        <f>ROUND(D22*0.2,0)</f>
-        <v/>
-      </c>
-      <c r="E23" s="686" t="n"/>
-      <c r="G23" s="690" t="n"/>
-      <c r="H23" s="690" t="n"/>
-    </row>
-    <row r="24" hidden="1" s="373">
-      <c r="B24" s="340" t="n">
-        <v>7</v>
-      </c>
-      <c r="C24" s="340" t="inlineStr">
-        <is>
-          <t>Thuế TNDN quý 1.2024</t>
-        </is>
-      </c>
-      <c r="D24" s="688" t="n"/>
-      <c r="H24" s="695" t="n"/>
-    </row>
-    <row r="25" hidden="1" s="373">
-      <c r="B25" s="340" t="n">
-        <v>8</v>
-      </c>
-      <c r="C25" s="340" t="inlineStr">
-        <is>
-          <t>Thuế TNDN Quý 2.2024</t>
-        </is>
-      </c>
-      <c r="D25" s="688" t="n"/>
-      <c r="E25" s="693" t="n"/>
-      <c r="F25" s="693" t="n"/>
-    </row>
-    <row r="26" hidden="1" s="373">
-      <c r="B26" s="340" t="n">
-        <v>9</v>
-      </c>
-      <c r="C26" s="340" t="inlineStr">
-        <is>
-          <t>Thuế TNDN quý 3.2024</t>
-        </is>
-      </c>
-      <c r="D26" s="688" t="n"/>
-      <c r="E26" s="693" t="n"/>
-      <c r="F26" s="693" t="n"/>
-    </row>
-    <row r="27" hidden="1" s="373">
-      <c r="B27" s="340" t="n">
-        <v>10</v>
-      </c>
-      <c r="C27" s="340" t="inlineStr">
-        <is>
-          <t>Thuế TNDN quý 4.2024</t>
-        </is>
-      </c>
-      <c r="D27" s="696">
-        <f>D23-D24-D25-D26</f>
-        <v/>
-      </c>
-      <c r="E27" s="693" t="n"/>
-      <c r="F27" s="693" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="340" t="n">
-        <v>7</v>
-      </c>
-      <c r="C28" s="340" t="inlineStr">
-        <is>
-          <t>Lợi nhuận trước thuế</t>
-        </is>
-      </c>
-      <c r="D28" s="688">
-        <f>D7-D11</f>
-        <v/>
-      </c>
-      <c r="E28" s="693" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="340" t="n">
-        <v>8</v>
-      </c>
-      <c r="C29" s="340" t="inlineStr">
-        <is>
-          <t>Lợi nhuận sau thuế Quý 1 năm 2026</t>
-        </is>
-      </c>
-      <c r="D29" s="688">
-        <f>D28-D23</f>
-        <v/>
-      </c>
-      <c r="E29" s="693" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="352" t="n"/>
-      <c r="C30" s="352" t="n"/>
-      <c r="D30" s="686" t="n"/>
-      <c r="E30" s="693" t="n"/>
-      <c r="F30" s="693" t="n"/>
-      <c r="G30" s="697" t="n"/>
-      <c r="H30" s="697" t="n"/>
-    </row>
-    <row r="31">
-      <c r="B31" s="525" t="inlineStr">
-        <is>
-          <t>Lập bảng                                         Kiểm soát                                              Tổng giám đốc</t>
-        </is>
-      </c>
-      <c r="H31" s="697" t="n"/>
-    </row>
-    <row r="32">
-      <c r="F32" s="690" t="n"/>
-    </row>
-    <row r="33">
-      <c r="F33" s="697" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="A4:D4"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet2">
     <tabColor theme="3" tint="0.7999816888943144"/>
@@ -13731,7 +14587,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet3">
     <tabColor theme="3" tint="0.7999816888943144"/>
@@ -13750,7 +14606,7 @@
     <col hidden="1" width="41.42578125" customWidth="1" style="578" min="11" max="11"/>
     <col hidden="1" width="41.42578125" customWidth="1" style="18" min="12" max="12"/>
     <col hidden="1" width="17.28515625" customWidth="1" style="18" min="13" max="13"/>
-    <col hidden="1" style="18" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" style="18" min="14" max="14"/>
     <col width="41.42578125" customWidth="1" style="18" min="15" max="16384"/>
   </cols>
   <sheetData>
@@ -16983,7 +17839,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet4">
     <tabColor theme="3" tint="0.7999816888943144"/>
@@ -20482,7 +21338,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet5">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21379,7 +22235,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet7">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22285,7 +23141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet8">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -29721,7 +30577,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet9">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -30211,410 +31067,4 @@
   <pageSetup orientation="portrait"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet10">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" style="292" min="1" max="2"/>
-    <col width="10" customWidth="1" style="373" min="3" max="3"/>
-    <col width="29.28515625" bestFit="1" customWidth="1" style="373" min="4" max="4"/>
-    <col width="9.140625" customWidth="1" style="373" min="5" max="6"/>
-    <col width="14" bestFit="1" customWidth="1" style="315" min="7" max="7"/>
-    <col width="11.42578125" bestFit="1" customWidth="1" style="294" min="8" max="8"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" style="315" min="9" max="9"/>
-    <col width="11.42578125" bestFit="1" customWidth="1" style="294" min="10" max="10"/>
-    <col width="5.42578125" bestFit="1" customWidth="1" style="315" min="11" max="11"/>
-    <col width="5.5703125" bestFit="1" customWidth="1" style="294" min="12" max="12"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" style="315" min="13" max="13"/>
-    <col width="11.42578125" bestFit="1" customWidth="1" style="294" min="14" max="14"/>
-    <col width="13.5703125" customWidth="1" style="373" min="15" max="15"/>
-    <col width="18.140625" customWidth="1" style="373" min="16" max="16"/>
-    <col width="8.7109375" customWidth="1" style="373" min="17" max="16384"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18.75" customHeight="1" s="373">
-      <c r="A1" s="516" t="inlineStr">
-        <is>
-          <t>SỔ CHI TIẾT CÁC TÀI KHOẢN</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="517" t="inlineStr">
-        <is>
-          <t>Loại tiền: Tổng hợp; Tài khoản: 421; Quý 1 năm 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16.5" customHeight="1" s="373">
-      <c r="A3" s="522" t="inlineStr">
-        <is>
-          <t>Ngày hạch toán</t>
-        </is>
-      </c>
-      <c r="B3" s="522" t="inlineStr">
-        <is>
-          <t>Ngày chứng từ</t>
-        </is>
-      </c>
-      <c r="C3" s="518" t="inlineStr">
-        <is>
-          <t>Số chứng từ</t>
-        </is>
-      </c>
-      <c r="D3" s="518" t="inlineStr">
-        <is>
-          <t>Diễn giải</t>
-        </is>
-      </c>
-      <c r="E3" s="518" t="inlineStr">
-        <is>
-          <t>Tài khoản</t>
-        </is>
-      </c>
-      <c r="F3" s="518" t="inlineStr">
-        <is>
-          <t>TK đối ứng</t>
-        </is>
-      </c>
-      <c r="G3" s="683" t="inlineStr">
-        <is>
-          <t>Phát sinh Nợ</t>
-        </is>
-      </c>
-      <c r="H3" s="684" t="n"/>
-      <c r="I3" s="683" t="inlineStr">
-        <is>
-          <t>Phát sinh Có</t>
-        </is>
-      </c>
-      <c r="J3" s="684" t="n"/>
-      <c r="K3" s="683" t="inlineStr">
-        <is>
-          <t>Dư Nợ</t>
-        </is>
-      </c>
-      <c r="L3" s="684" t="n"/>
-      <c r="M3" s="683" t="inlineStr">
-        <is>
-          <t>Dư Có</t>
-        </is>
-      </c>
-      <c r="N3" s="684" t="n"/>
-      <c r="O3" s="518" t="inlineStr">
-        <is>
-          <t>Mã mục thu/chi</t>
-        </is>
-      </c>
-      <c r="P3" s="518" t="inlineStr">
-        <is>
-          <t>Tên mục thu/chi</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="373">
-      <c r="A4" s="685" t="n"/>
-      <c r="B4" s="685" t="n"/>
-      <c r="C4" s="685" t="n"/>
-      <c r="D4" s="685" t="n"/>
-      <c r="E4" s="685" t="n"/>
-      <c r="F4" s="685" t="n"/>
-      <c r="G4" s="376" t="inlineStr">
-        <is>
-          <t>Số tiền</t>
-        </is>
-      </c>
-      <c r="H4" s="377" t="inlineStr">
-        <is>
-          <t>Quy đổi</t>
-        </is>
-      </c>
-      <c r="I4" s="376" t="inlineStr">
-        <is>
-          <t>Số tiền</t>
-        </is>
-      </c>
-      <c r="J4" s="377" t="inlineStr">
-        <is>
-          <t>Quy đổi</t>
-        </is>
-      </c>
-      <c r="K4" s="376" t="inlineStr">
-        <is>
-          <t>Số tiền</t>
-        </is>
-      </c>
-      <c r="L4" s="377" t="inlineStr">
-        <is>
-          <t>Quy đổi</t>
-        </is>
-      </c>
-      <c r="M4" s="376" t="inlineStr">
-        <is>
-          <t>Số tiền</t>
-        </is>
-      </c>
-      <c r="N4" s="377" t="inlineStr">
-        <is>
-          <t>Quy đổi</t>
-        </is>
-      </c>
-      <c r="O4" s="685" t="n"/>
-      <c r="P4" s="685" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="378" t="n"/>
-      <c r="B5" s="378" t="n"/>
-      <c r="C5" s="379" t="inlineStr"/>
-      <c r="D5" s="379" t="inlineStr">
-        <is>
-          <t>Số dư đầu kỳ</t>
-        </is>
-      </c>
-      <c r="E5" s="379" t="inlineStr">
-        <is>
-          <t>421</t>
-        </is>
-      </c>
-      <c r="F5" s="379" t="n"/>
-      <c r="G5" s="380" t="n"/>
-      <c r="H5" s="381" t="n"/>
-      <c r="I5" s="380" t="n"/>
-      <c r="J5" s="381" t="n"/>
-      <c r="K5" s="380" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="381" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="380" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="N5" s="381" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="O5" s="379" t="n"/>
-      <c r="P5" s="379" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="378" t="n">
-        <v>46027</v>
-      </c>
-      <c r="B6" s="378" t="n">
-        <v>46027</v>
-      </c>
-      <c r="C6" s="379" t="inlineStr">
-        <is>
-          <t>ZKC01</t>
-        </is>
-      </c>
-      <c r="D6" s="379" t="inlineStr">
-        <is>
-          <t>Kết chuyển lợi nhuận sau thuế năm 2025</t>
-        </is>
-      </c>
-      <c r="E6" s="379" t="inlineStr">
-        <is>
-          <t>421</t>
-        </is>
-      </c>
-      <c r="F6" s="379" t="inlineStr">
-        <is>
-          <t>42121.01</t>
-        </is>
-      </c>
-      <c r="G6" s="380" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="381" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="380" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="J6" s="381" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="K6" s="380" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="381" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="380" t="n">
-        <v>35934868090</v>
-      </c>
-      <c r="N6" s="381" t="n">
-        <v>35934868090</v>
-      </c>
-      <c r="O6" s="379" t="n"/>
-      <c r="P6" s="379" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="378" t="n">
-        <v>46027</v>
-      </c>
-      <c r="B7" s="378" t="n">
-        <v>46027</v>
-      </c>
-      <c r="C7" s="379" t="inlineStr">
-        <is>
-          <t>ZKC01</t>
-        </is>
-      </c>
-      <c r="D7" s="379" t="inlineStr">
-        <is>
-          <t>Kết chuyển lợi nhuận sau thuế năm 2025</t>
-        </is>
-      </c>
-      <c r="E7" s="379" t="inlineStr">
-        <is>
-          <t>421</t>
-        </is>
-      </c>
-      <c r="F7" s="379" t="inlineStr">
-        <is>
-          <t>42111.01</t>
-        </is>
-      </c>
-      <c r="G7" s="380" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="H7" s="381" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="I7" s="380" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="381" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="380" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="381" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="380" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="N7" s="381" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="O7" s="379" t="n"/>
-      <c r="P7" s="379" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="378" t="n"/>
-      <c r="B8" s="378" t="n"/>
-      <c r="C8" s="379" t="inlineStr"/>
-      <c r="D8" s="379" t="inlineStr">
-        <is>
-          <t>Cộng</t>
-        </is>
-      </c>
-      <c r="E8" s="379" t="inlineStr">
-        <is>
-          <t>421</t>
-        </is>
-      </c>
-      <c r="F8" s="379" t="n"/>
-      <c r="G8" s="380" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="H8" s="381" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="I8" s="380" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="J8" s="381" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="K8" s="380" t="n"/>
-      <c r="L8" s="381" t="n"/>
-      <c r="M8" s="380" t="n"/>
-      <c r="N8" s="381" t="n"/>
-      <c r="O8" s="379" t="n"/>
-      <c r="P8" s="379" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="378" t="n"/>
-      <c r="B9" s="378" t="n"/>
-      <c r="C9" s="379" t="inlineStr"/>
-      <c r="D9" s="379" t="inlineStr">
-        <is>
-          <t>Số dư cuối kỳ</t>
-        </is>
-      </c>
-      <c r="E9" s="379" t="inlineStr">
-        <is>
-          <t>421</t>
-        </is>
-      </c>
-      <c r="F9" s="379" t="n"/>
-      <c r="G9" s="380" t="n"/>
-      <c r="H9" s="381" t="n"/>
-      <c r="I9" s="380" t="n"/>
-      <c r="J9" s="381" t="n"/>
-      <c r="K9" s="380" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="381" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="380" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="N9" s="381" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="O9" s="379" t="n"/>
-      <c r="P9" s="379" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="382" t="inlineStr">
-        <is>
-          <t>Số dòng = 5</t>
-        </is>
-      </c>
-      <c r="G10" s="383" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="H10" s="384" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="I10" s="383" t="n">
-        <v>17967434045</v>
-      </c>
-      <c r="J10" s="384" t="n">
-        <v>17967434045</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="O3:O4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="M3:N3"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="I3:J3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>